<commit_message>
Add zero-mark and page-number safeguards
</commit_message>
<xml_diff>
--- a/DCA Script Marker — DCA State Template.xlsx
+++ b/DCA Script Marker — DCA State Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R7d9fbc22dbb44a70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character List" sheetId="3" r:id="Rcfe097052ded4c04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCA States" sheetId="1" r:id="R3d85b9df19114afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R2bcb9c7fe78a4d0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character List" sheetId="3" r:id="R192aa10882ce4700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCA States" sheetId="1" r:id="R81ca3d08d97f4814"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,14 +95,6 @@
     <x:t xml:space="preserve">Page Hint</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Optional page number to help locate the correct cue when the same text appears more than once.
-填入剧本页码来帮助更好的找到这段文字提示。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use the page number printed inside the script whenever it is available. If the script does not show an internal page number, enter the PDF page number instead.
-如剧本页面内印有页码，请填写该剧本内部页码；如剧本没有内部页码，请填写 PDF 页码。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">DCA cells</x:t>
   </x:si>
   <x:si>
@@ -134,9 +126,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Type each character name from here</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">One row = one DCA State. Keep start cue, position, and page hint separate; use a new line for each person in a DCA cell.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">DCA 1</x:t>
@@ -746,23 +735,25 @@
       </x:c>
       <x:c r="C13" s="1"/>
     </x:row>
-    <x:row r="14" ht="75">
+    <x:row r="14" ht="105" customHeight="1">
       <x:c r="A14" s="11" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="s">
+      <x:c r="B14" s="1" t="str">
+        <x:v>Optional. Use when the same cue text appears more than once.
+可选。同一提示文字重复出现时使用。</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Use the page number printed inside the script. If none is printed, use the sequential PDF page position shown by the viewer (cover = PDF page 1). Do not confuse this with the app's selected-page range, which always uses PDF page positions.
+填写剧本页面内印刷的页码；如果没有印刷页码，再填写 PDF 阅读器显示的顺序页码（封面 = PDF 第 1 页）。不要与软件中的指定页码范围混用；该范围始终使用 PDF 顺序页码。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="105">
+      <x:c r="A15" s="11" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="C14" s="1" t="s">
+      <x:c r="B15" s="1" t="s">
         <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="105">
-      <x:c r="A15" s="11" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B15" s="1" t="s">
-        <x:v>27</x:v>
       </x:c>
       <x:c r="C15" s="1"/>
     </x:row>
@@ -786,29 +777,29 @@
   <x:sheetData>
     <x:row r="1" ht="18">
       <x:c r="A1" s="18" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="160">
+      <x:c r="A2" s="19" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="s">
+      <x:c r="B2" s="14" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="160">
-      <x:c r="A2" s="19" t="s">
+      <x:c r="C2" s="14" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B2" s="14" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="C2" s="14" t="s">
-        <x:v>32</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" ht="16">
       <x:c r="A3" s="20" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="16">
@@ -1861,9 +1852,9 @@
       <x:c r="Q1" s="25"/>
       <x:c r="R1" s="25"/>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="26" t="s">
-        <x:v>34</x:v>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="26" t="str">
+        <x:v>Page Hint = printed script page; if none is printed, use the PDF page position. Selected-page ranges in the app always use PDF page positions. / Page Hint = 剧本内印刷页码；没有印刷页码时才使用 PDF 顺序页码。软件中的指定页码范围始终使用 PDF 顺序页码。</x:v>
       </x:c>
       <x:c r="B2" s="26"/>
       <x:c r="C2" s="26"/>
@@ -1900,43 +1891,43 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="F4" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G4" s="9" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I4" s="9" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="J4" s="9" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="H4" s="9" t="s">
+      <x:c r="K4" s="9" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="s">
+      <x:c r="L4" s="9" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="J4" s="9" t="s">
+      <x:c r="M4" s="9" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="K4" s="9" t="s">
+      <x:c r="N4" s="9" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="L4" s="9" t="s">
+      <x:c r="O4" s="9" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="M4" s="9" t="s">
+      <x:c r="P4" s="9" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="N4" s="9" t="s">
+      <x:c r="Q4" s="9" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="O4" s="9" t="s">
+      <x:c r="R4" s="9" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="P4" s="9" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="Q4" s="9" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="R4" s="9" t="s">
-        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" customHeight="1">

</xml_diff>